<commit_message>
Removed Additional Info column from Admin Registrations table, server processing, and registration form
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,42 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="006B0F2A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDF5E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -68,52 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D4A843"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D4A843"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D4A843"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D4A843"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00E0C080"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E0C080"/>
-      </right>
-      <top style="thin">
-        <color rgb="00E0C080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E0C080"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -479,163 +413,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>S.No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Reg. ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Event</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>College</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Participant 1 Name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Participant 1 Email</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Participant 2 Name</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Participant 2 Email</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Additional Info</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Registered On</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Check-In Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Check-In Time</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>DV26-PTD-OO5TM</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Pitch The Deck</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>SRM</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Data science</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>kathir</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>abijosboo@gmail.com</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Vimal</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>abijosvimalpalsam2000@gmail.com</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Machine Learning</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>01-08-2026 09:07</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>Checked In</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>01-08-2026 09:07:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fully updated all events, venues, timings, coordinators, and replaced Mega Auction with Pitch Perfect as per new PDF
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -26,15 +26,25 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDF5E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +52,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E0C080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E0C080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0C080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0C080"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,6 +510,71 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Check-In Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>DV26-PTD-FOYUL</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Pitch The Deck</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>SRM</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Data science</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Abijos</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>abijosboo@gmail.com</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>kathir</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>abijosvimalpalsam2000@gmail.com</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>01-08-2026 12:49</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Checked In</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>01-08-2026 12:50:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed list indices error by adding type check safeguards in leaderboard data sync
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,71 +510,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Check-In Time</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>DV26-PTD-FOYUL</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Pitch The Deck</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>SRM</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Data science</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>Abijos</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>abijosboo@gmail.com</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>kathir</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>abijosvimalpalsam2000@gmail.com</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>01-08-2026 12:49</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Checked In</t>
-        </is>
-      </c>
-      <c r="M2" s="1" t="inlineStr">
-        <is>
-          <t>01-08-2026 12:50:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed checkin lookup error handling and case-insensitivity
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,67 @@
           <t>Check-In Time</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>DV26-PPF-H32RH</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Plot Perfect</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>BCA</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>JENCY</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>jency.t.work@gmail.com</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>JOJO</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>dharini@gmail.com</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>01-08-2026 17:29</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated admin.html login error guidance
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -567,12 +567,16 @@
           <t>01-08-2026 17:29</t>
         </is>
       </c>
-      <c r="L2" s="1" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="M2" s="1" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Checked In</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>01-08-2026 17:41:42</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fixed relative page links and added dual route aliases for hosting compatibility
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,71 +510,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Check-In Time</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>DV26-PPF-H32RH</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Plot Perfect</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>WCC</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>BCA</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>JENCY</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>jency.t.work@gmail.com</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>JOJO</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>dharini@gmail.com</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>01-08-2026 17:29</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Checked In</t>
-        </is>
-      </c>
-      <c r="M2" s="1" t="inlineStr">
-        <is>
-          <t>01-08-2026 17:41:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed Spot Registration save error and restricted Leaderboard display to Checked In students only
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -26,7 +26,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,12 +75,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -443,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +518,120 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Check-In Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>DV26-PTD-ISPXJ</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Pitch The Deck</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Test College</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Spot Tester</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>spottester@gmail.com</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr"/>
+      <c r="I2" s="1" t="inlineStr"/>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>04-08-2026 09:36</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Checked In</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>04-08-2026 09:36:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>DV26-PTD-CP1RJ</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Pitch The Deck</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Test College</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Spot Tester</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>spottester@gmail.com</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>04-08-2026 09:36</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Checked In</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>04-08-2026 09:36:53</t>
         </is>
       </c>
     </row>

</xml_diff>